<commit_message>
Updatting E-commerce project with new features and test cases for API, UI, and database validation. Added frontend pages and styles for a complete user experience.
</commit_message>
<xml_diff>
--- a/ecommerce_QA_master_test_cases.xlsx
+++ b/ecommerce_QA_master_test_cases.xlsx
@@ -6097,7 +6097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7386,7 +7386,6 @@
       <c r="H32" t="n">
         <v>0.03</v>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7427,7 +7426,6 @@
       <c r="H33" t="n">
         <v>0.01</v>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7468,7 +7466,6 @@
       <c r="H34" t="n">
         <v>0.02</v>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7509,7 +7506,6 @@
       <c r="H35" t="n">
         <v>0.03</v>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7550,7 +7546,6 @@
       <c r="H36" t="n">
         <v>0.03</v>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7591,7 +7586,6 @@
       <c r="H37" t="n">
         <v>0</v>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7632,7 +7626,6 @@
       <c r="H38" t="n">
         <v>0.01</v>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7673,7 +7666,6 @@
       <c r="H39" t="n">
         <v>0.01</v>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7714,7 +7706,6 @@
       <c r="H40" t="n">
         <v>0.01</v>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7755,7 +7746,6 @@
       <c r="H41" t="n">
         <v>0.01</v>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7796,7 +7786,6 @@
       <c r="H42" t="n">
         <v>0.01</v>
       </c>
-      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7837,7 +7826,6 @@
       <c r="H43" t="n">
         <v>0</v>
       </c>
-      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7878,7 +7866,6 @@
       <c r="H44" t="n">
         <v>0</v>
       </c>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -7919,7 +7906,6 @@
       <c r="H45" t="n">
         <v>0.01</v>
       </c>
-      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -7960,7 +7946,6 @@
       <c r="H46" t="n">
         <v>0</v>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -8001,7 +7986,6 @@
       <c r="H47" t="n">
         <v>0</v>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -8042,7 +8026,6 @@
       <c r="H48" t="n">
         <v>0</v>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -8083,7 +8066,6 @@
       <c r="H49" t="n">
         <v>0.02</v>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8124,7 +8106,6 @@
       <c r="H50" t="n">
         <v>0.03</v>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8165,7 +8146,6 @@
       <c r="H51" t="n">
         <v>0.01</v>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8206,7 +8186,6 @@
       <c r="H52" t="n">
         <v>0.01</v>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8247,7 +8226,6 @@
       <c r="H53" t="n">
         <v>0.36</v>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -8288,7 +8266,6 @@
       <c r="H54" t="n">
         <v>0.17</v>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8329,7 +8306,6 @@
       <c r="H55" t="n">
         <v>0.32</v>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8370,7 +8346,6 @@
       <c r="H56" t="n">
         <v>0.08</v>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8411,7 +8386,6 @@
       <c r="H57" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8452,7 +8426,3273 @@
       <c r="H58" t="n">
         <v>0.06</v>
       </c>
-      <c r="I58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TC-ORD-006</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>test_create_order_with_zero_quantity</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_zero_quantity</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TC-ORD-007</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>test_create_order_with_empty_items</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_empty_items</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TC-ORD-008</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>test_create_order_with_negative_quantity</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_negative_quantity</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TC-ORD-001</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>test_create_order</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TC-ORD-002</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>test_get_existing_order</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_get_existing_order</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TC-ORD-003</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_order</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_get_nonexistent_order</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TC-ORD-004</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>test_create_order_with_invalid_user</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order_with_invalid_user</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TC-ORD-005</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>test_create_order_with_invalid_product</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order_with_invalid_product</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TC-PROD-001</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>test_create_product</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TC-PROD-002</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>test_get_existing_product</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_get_existing_product</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TC-PROD-003</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_product</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_get_nonexistent_product</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>TC-PROD-004</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>test_create_product_missing_name</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product_missing_name</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TC-PROD-005</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>test_create_product_missing_category</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product_missing_category</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TC-USER-001</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>test_create_user</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>TC-USER-002</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_user</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_get_nonexistent_user</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TC-USER-003</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>test_create_user_with_invalid_email</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_with_invalid_email</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>TC-USER-004</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>test_create_user_missing_username</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_missing_username</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>TC-USER-005</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>test_create_user_with_duplicate_username</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_with_duplicate_username</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TC-DB-003</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>test_created_order_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>tests/db/test_orders_db.py::test_created_order_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>TC-DB-002</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>test_created_product_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>tests/db/test_products_db.py::test_created_product_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>TC-DB-001</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>test_created_user_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>tests/db/test_users_db.py::test_created_user_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>TC-E2E-001</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>test_complete_purchase_flow</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>tests/e2e/test_complete_purchase_flow.py::test_complete_purchase_flow</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>0.55</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>TC-UI-003</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>test_add_product_to_cart</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>tests/ui/test_cart_ui.py::test_add_product_to_cart</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H81" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>TC-UI-004</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>test_place_order_from_ui</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>tests/ui/test_checkout_ui.py::test_place_order_from_ui</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H82" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>TC-UI-005</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>test_empty_cart_cannot_checkout</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>tests/ui/test_empty_cart_ui.py::test_empty_cart_cannot_checkout</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H83" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>TC-UI-001</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>test_login_page_loads</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>tests/ui/test_login_ui.py::test_login_page_loads</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H84" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>TC-UI-002</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>test_products_page_displays_products</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>tests/ui/test_products_ui.py::test_products_page_displays_products</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H85" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>TC-ORD-006</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>test_create_order_with_zero_quantity</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_zero_quantity</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H86" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>TC-ORD-007</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>test_create_order_with_empty_items</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_empty_items</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H87" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>TC-ORD-008</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>test_create_order_with_negative_quantity</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_negative_quantity</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>TC-ORD-001</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>test_create_order</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>TC-ORD-002</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>test_get_existing_order</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_get_existing_order</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H90" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>TC-ORD-003</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_order</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_get_nonexistent_order</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H91" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>TC-ORD-004</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>test_create_order_with_invalid_user</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order_with_invalid_user</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H92" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>TC-ORD-005</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>test_create_order_with_invalid_product</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order_with_invalid_product</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H93" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>TC-PROD-001</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>test_create_product</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H94" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>TC-PROD-002</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>test_get_existing_product</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_get_existing_product</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H95" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>TC-PROD-003</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_product</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_get_nonexistent_product</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H96" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>TC-PROD-004</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>test_create_product_missing_name</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product_missing_name</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>TC-PROD-005</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>test_create_product_missing_category</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product_missing_category</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>TC-USER-001</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>test_create_user</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H99" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>TC-USER-002</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_user</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_get_nonexistent_user</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H100" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>TC-USER-003</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>test_create_user_with_invalid_email</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_with_invalid_email</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H101" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>TC-USER-004</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>test_create_user_missing_username</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_missing_username</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>TC-USER-005</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>test_create_user_with_duplicate_username</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_with_duplicate_username</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H103" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>TC-DB-003</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>test_created_order_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>tests/db/test_orders_db.py::test_created_order_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H104" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>TC-DB-002</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>test_created_product_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>tests/db/test_products_db.py::test_created_product_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H105" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>TC-DB-001</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>test_created_user_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>tests/db/test_users_db.py::test_created_user_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H106" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>TC-E2E-001</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>test_complete_purchase_flow</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>tests/e2e/test_complete_purchase_flow.py::test_complete_purchase_flow</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H107" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>TC-UI-003</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>test_add_product_to_cart</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>tests/ui/test_cart_ui.py::test_add_product_to_cart</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>TC-UI-004</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>test_place_order_from_ui</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>tests/ui/test_checkout_ui.py::test_place_order_from_ui</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H109" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>TC-UI-005</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>test_empty_cart_cannot_checkout</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>tests/ui/test_empty_cart_ui.py::test_empty_cart_cannot_checkout</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H110" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>TC-UI-001</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>test_login_page_loads</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>tests/ui/test_login_ui.py::test_login_page_loads</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>TC-UI-002</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>test_products_page_displays_products</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>tests/ui/test_products_ui.py::test_products_page_displays_products</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H112" t="n">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>TC-ORD-006</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>test_create_order_with_zero_quantity</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_zero_quantity</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H113" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>TC-ORD-007</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>test_create_order_with_empty_items</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_empty_items</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H114" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>TC-ORD-008</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>test_create_order_with_negative_quantity</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>tests/api/test_order_validation_api.py::test_create_order_with_negative_quantity</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H115" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>TC-ORD-001</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>test_create_order</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H116" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>TC-ORD-002</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>test_get_existing_order</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_get_existing_order</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H117" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>TC-ORD-003</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_order</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_get_nonexistent_order</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H118" t="n">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>TC-ORD-004</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>test_create_order_with_invalid_user</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order_with_invalid_user</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H119" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>TC-ORD-005</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>test_create_order_with_invalid_product</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>tests/api/test_orders_api.py::test_create_order_with_invalid_product</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H120" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>TC-PROD-001</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>test_create_product</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H121" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>TC-PROD-002</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>test_get_existing_product</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_get_existing_product</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H122" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>TC-PROD-003</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_product</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_get_nonexistent_product</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H123" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>TC-PROD-004</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>test_create_product_missing_name</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product_missing_name</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>TC-PROD-005</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>test_create_product_missing_category</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>tests/api/test_products_api.py::test_create_product_missing_category</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>TC-USER-001</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>test_create_user</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H126" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>TC-USER-002</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>test_get_nonexistent_user</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_get_nonexistent_user</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H127" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>TC-USER-003</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>test_create_user_with_invalid_email</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_with_invalid_email</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>TC-USER-004</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>test_create_user_missing_username</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_missing_username</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>TC-USER-005</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>test_create_user_with_duplicate_username</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>tests/api/test_users_api.py::test_create_user_with_duplicate_username</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H130" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>TC-DB-003</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>test_created_order_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>tests/db/test_orders_db.py::test_created_order_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H131" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>TC-DB-002</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>test_created_product_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>tests/db/test_products_db.py::test_created_product_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H132" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>TC-DB-001</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>test_created_user_exists_in_database</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>tests/db/test_users_db.py::test_created_user_exists_in_database</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H133" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>TC-E2E-001</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>test_complete_purchase_flow</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>tests/e2e/test_complete_purchase_flow.py::test_complete_purchase_flow</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H134" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>TC-UI-003</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>test_add_product_to_cart</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>tests/ui/test_cart_ui.py::test_add_product_to_cart</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H135" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="I135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>TC-UI-004</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>test_place_order_from_ui</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>tests/ui/test_checkout_ui.py::test_place_order_from_ui</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H136" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>TC-UI-005</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>test_empty_cart_cannot_checkout</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>tests/ui/test_empty_cart_ui.py::test_empty_cart_cannot_checkout</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H137" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>TC-UI-001</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>test_login_page_loads</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>tests/ui/test_login_ui.py::test_login_page_loads</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H138" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>TC-UI-002</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>test_products_page_displays_products</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>tests/ui/test_products_ui.py::test_products_page_displays_products</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="H139" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I139" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8465,7 +11705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8670,6 +11910,102 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021639</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>02:16:43</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>27</v>
+      </c>
+      <c r="E7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021650</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>02:16:54</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>27</v>
+      </c>
+      <c r="E8" t="n">
+        <v>27</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RUN-20260930-021910</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>02:19:13</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>27</v>
+      </c>
+      <c r="E9" t="n">
+        <v>27</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>